<commit_message>
docs(shared): add bilingual presentation decks and demo cleanup documentation
</commit_message>
<xml_diff>
--- a/Shared/academia-demo-cleanup-plan.xlsx
+++ b/Shared/academia-demo-cleanup-plan.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Endpoints الباك اند" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="مشاكل حرجة بالباك اند" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تدقيق الحقول والـPagination" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الصفحات العامة (Landing)" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'حالة الصفحات (قبل وبعد)'!$A$1:$G$31</definedName>
@@ -126,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -183,6 +184,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -549,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -680,11 +684,89 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>ملاحظات UI متفرقة تم تنفيذها</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>• إصلاح خط العناوين بالإنجليزي (كان Reem Kufi -خط كوفي عربي الطابع- بالغلط، صار Poppins محمّل فعلياً بـGoogle Fonts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>• إصلاح تباين خلفية السايدبار مع كلمة Academia بوضع النهار</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>• توحيد حجم/وزن خط 'Academia' بالشريط العلوي للموبايل مع نسخة السايدبار</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>• قفل سكرول محتوى الصفحة خلف الأوفرلاي أثناء فتح القائمة الجانبية بالموبايل</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>• إعادة تنظيم القائمة الجانبية للأدمن (وحدة واحدة بدل اثنتين، بلا مجلدات لعنصر واحد)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>تنظيف القائمة الجانبية لكل الأدوار</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>• الطالب: حُذف مجلّدان بعنصر واحد (أدوات الدراسة / التقدّم والجدول) → كورساتي، الجدول، محفظتي بأعلى المستوى</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>• المعلم: حُذف مجلّد التدريس بعنصر واحد → كورساتي والأرباح بأعلى المستوى؛ بقي مجلّد 'ملفي المهني' (عنصران)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>• ولي الأمر: مسطّحة أصلاً؛ الأدمن: وحدة واحدة (رُتّبت سابقاً)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="11">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A19:F19"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A20:F20"/>
+    <mergeCell ref="A21:F21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -746,7 +828,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>الإدارة</t>
         </is>
@@ -756,7 +838,7 @@
           <t>وحدات النظام</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="15" t="inlineStr">
         <is>
           <t>ديمو/وهمية</t>
         </is>
@@ -783,7 +865,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>الإدارة</t>
         </is>
@@ -793,7 +875,7 @@
           <t>أنواع المستخدم/الأدوار</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>ديمو/وهمية</t>
         </is>
@@ -820,7 +902,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>الإدارة</t>
         </is>
@@ -830,7 +912,7 @@
           <t>مصفوفة الصلاحيات (rbac قديمة)</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>ديمو/وهمية</t>
         </is>
@@ -857,7 +939,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>الإدارة</t>
         </is>
@@ -867,7 +949,7 @@
           <t>المنهاج الأكاديمي</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>ديمو/وهمية</t>
         </is>
@@ -894,7 +976,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>الإدارة</t>
         </is>
@@ -904,7 +986,7 @@
           <t>طلبات المنهاج</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>ديمو/وهمية</t>
         </is>
@@ -931,7 +1013,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>الإدارة</t>
         </is>
@@ -941,7 +1023,7 @@
           <t>مراجعة المحتوى</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="15" t="inlineStr">
         <is>
           <t>ديمو/وهمية</t>
         </is>
@@ -968,7 +1050,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>الإدارة</t>
         </is>
@@ -978,7 +1060,7 @@
           <t>بلاغات المجتمع</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="15" t="inlineStr">
         <is>
           <t>ديمو/وهمية</t>
         </is>
@@ -1005,7 +1087,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>الإدارة</t>
         </is>
@@ -1015,7 +1097,7 @@
           <t>توثيق المعلمين</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>ديمو/وهمية</t>
         </is>
@@ -1042,7 +1124,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>الإدارة</t>
         </is>
@@ -1052,12 +1134,12 @@
           <t>لوحة إدارة Academia</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="15" t="inlineStr">
         <is>
           <t>ديمو/وهمية بالكامل</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
+      <c r="D10" s="16" t="inlineStr">
         <is>
           <t>حقيقية 100% + موسّعة</t>
         </is>
@@ -1079,7 +1161,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>الإدارة</t>
         </is>
@@ -1089,12 +1171,12 @@
           <t>صلاحيات الباك اند</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <t>حقيقية أصلاً</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D11" s="15" t="inlineStr">
         <is>
           <t>حقيقية (بلا تغيير جوهري)</t>
         </is>
@@ -1116,7 +1198,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>الإدارة</t>
         </is>
@@ -1126,12 +1208,12 @@
           <t>الصفحات (Pages)</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <t>حقيقية أصلاً</t>
         </is>
       </c>
-      <c r="D12" s="11" t="inlineStr">
+      <c r="D12" s="16" t="inlineStr">
         <is>
           <t>حقيقية (بلا تغيير)</t>
         </is>
@@ -1153,7 +1235,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>الإدارة</t>
         </is>
@@ -1163,12 +1245,12 @@
           <t>الثوابت (Constants)</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C13" s="15" t="inlineStr">
         <is>
           <t>حقيقية أصلاً</t>
         </is>
       </c>
-      <c r="D13" s="11" t="inlineStr">
+      <c r="D13" s="16" t="inlineStr">
         <is>
           <t>حقيقية (بلا تغيير)</t>
         </is>
@@ -1190,7 +1272,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>الإدارة</t>
         </is>
@@ -1200,12 +1282,12 @@
           <t>المستخدمون</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <t>حقيقية أصلاً</t>
         </is>
       </c>
-      <c r="D14" s="11" t="inlineStr">
+      <c r="D14" s="16" t="inlineStr">
         <is>
           <t>حقيقية (بلا تغيير)</t>
         </is>
@@ -1227,7 +1309,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>الإدارة</t>
         </is>
@@ -1237,12 +1319,12 @@
           <t>المدفوعات (Wallet)</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C15" s="15" t="inlineStr">
         <is>
           <t>حقيقية أصلاً</t>
         </is>
       </c>
-      <c r="D15" s="11" t="inlineStr">
+      <c r="D15" s="16" t="inlineStr">
         <is>
           <t>حقيقية (بلا تغيير)</t>
         </is>
@@ -1264,7 +1346,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>الإدارة</t>
         </is>
@@ -1274,12 +1356,12 @@
           <t>كتالوج الكورسات</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C16" s="15" t="inlineStr">
         <is>
           <t>ديمو/وهمية بالكامل</t>
         </is>
       </c>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="D16" s="17" t="inlineStr">
         <is>
           <t>حقيقية 100% (عرض)، إنشاء معطّل بقصد</t>
         </is>
@@ -1301,7 +1383,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>عام</t>
         </is>
@@ -1311,7 +1393,7 @@
           <t>مساحة «المشرف» بالكامل (4 صفحات)</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C17" s="15" t="inlineStr">
         <is>
           <t>ديمو/وهمية</t>
         </is>
@@ -1338,7 +1420,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="15" t="inlineStr">
         <is>
           <t>الطالب</t>
         </is>
@@ -1348,12 +1430,12 @@
           <t>لوحة الطالب</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C18" s="15" t="inlineStr">
         <is>
           <t>ديمو/وهمية</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
+      <c r="D18" s="16" t="inlineStr">
         <is>
           <t>حقيقية 100%</t>
         </is>
@@ -1375,7 +1457,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>الطالب</t>
         </is>
@@ -1385,12 +1467,12 @@
           <t>كورساتي</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C19" s="15" t="inlineStr">
         <is>
           <t>ديمو/وهمية</t>
         </is>
       </c>
-      <c r="D19" s="11" t="inlineStr">
+      <c r="D19" s="16" t="inlineStr">
         <is>
           <t>حقيقية 100%</t>
         </is>
@@ -1412,7 +1494,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>الطالب</t>
         </is>
@@ -1422,12 +1504,12 @@
           <t>الجدول</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C20" s="15" t="inlineStr">
         <is>
           <t>ديمو/وهمية</t>
         </is>
       </c>
-      <c r="D20" s="11" t="inlineStr">
+      <c r="D20" s="16" t="inlineStr">
         <is>
           <t>حقيقية 100%</t>
         </is>
@@ -1449,7 +1531,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>الطالب</t>
         </is>
@@ -1459,12 +1541,12 @@
           <t>الإشعارات</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C21" s="15" t="inlineStr">
         <is>
           <t>ديمو/وهمية</t>
         </is>
       </c>
-      <c r="D21" s="12" t="inlineStr">
+      <c r="D21" s="17" t="inlineStr">
         <is>
           <t>حقيقية للطالب فقط</t>
         </is>
@@ -1486,7 +1568,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>الطالب</t>
         </is>
@@ -1496,7 +1578,7 @@
           <t>المكتبة/البطاقات/الاختبارات التجريبية/بنك الأخطاء/المفضلة/الإنجازات/شهاداتي/أسئلتي/الإحالات (9 صفحات)</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C22" s="15" t="inlineStr">
         <is>
           <t>ديمو/وهمية</t>
         </is>
@@ -1523,7 +1605,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t>الطالب</t>
         </is>
@@ -1533,12 +1615,12 @@
           <t>محفظتي</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
+      <c r="C23" s="15" t="inlineStr">
         <is>
           <t>حقيقية أصلاً</t>
         </is>
       </c>
-      <c r="D23" s="11" t="inlineStr">
+      <c r="D23" s="16" t="inlineStr">
         <is>
           <t>حقيقية (بلا تغيير)</t>
         </is>
@@ -1560,7 +1642,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="inlineStr">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>المعلم</t>
         </is>
@@ -1570,12 +1652,12 @@
           <t>لوحة المعلم</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="C24" s="15" t="inlineStr">
         <is>
           <t>ديمو/وهمية</t>
         </is>
       </c>
-      <c r="D24" s="12" t="inlineStr">
+      <c r="D24" s="17" t="inlineStr">
         <is>
           <t>حقيقية جزئياً (رصيد المحفظة)</t>
         </is>
@@ -1597,7 +1679,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="inlineStr">
+      <c r="A25" s="15" t="inlineStr">
         <is>
           <t>المعلم</t>
         </is>
@@ -1607,12 +1689,12 @@
           <t>كورساتي (معلم)</t>
         </is>
       </c>
-      <c r="C25" s="8" t="inlineStr">
+      <c r="C25" s="15" t="inlineStr">
         <is>
           <t>ديمو/وهمية</t>
         </is>
       </c>
-      <c r="D25" s="12" t="inlineStr">
+      <c r="D25" s="17" t="inlineStr">
         <is>
           <t>قيد تطوير — Placeholder موثّق</t>
         </is>
@@ -1634,7 +1716,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="inlineStr">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t>المعلم</t>
         </is>
@@ -1644,12 +1726,12 @@
           <t>تعديل ملفي</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr">
+      <c r="C26" s="15" t="inlineStr">
         <is>
           <t>ديمو/وهمية</t>
         </is>
       </c>
-      <c r="D26" s="12" t="inlineStr">
+      <c r="D26" s="17" t="inlineStr">
         <is>
           <t>حقيقية وظيفياً + تدهور رشيق</t>
         </is>
@@ -1671,7 +1753,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="inlineStr">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t>المعلم</t>
         </is>
@@ -1681,12 +1763,12 @@
           <t>الإعدادات (توفّر)</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
+      <c r="C27" s="15" t="inlineStr">
         <is>
           <t>ديمو/وهمية</t>
         </is>
       </c>
-      <c r="D27" s="12" t="inlineStr">
+      <c r="D27" s="17" t="inlineStr">
         <is>
           <t>حقيقية وظيفياً + تدهور رشيق</t>
         </is>
@@ -1708,7 +1790,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+      <c r="A28" s="15" t="inlineStr">
         <is>
           <t>المعلم</t>
         </is>
@@ -1718,12 +1800,12 @@
           <t>الأرباح</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
+      <c r="C28" s="15" t="inlineStr">
         <is>
           <t>حقيقية أصلاً</t>
         </is>
       </c>
-      <c r="D28" s="11" t="inlineStr">
+      <c r="D28" s="16" t="inlineStr">
         <is>
           <t>حقيقية (بلا تغيير)</t>
         </is>
@@ -1745,7 +1827,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="inlineStr">
+      <c r="A29" s="15" t="inlineStr">
         <is>
           <t>المعلم</t>
         </is>
@@ -1755,7 +1837,7 @@
           <t>المحتوى/الاختبارات/التصحيح/التحليلات/المجتمع (5 صفحات)</t>
         </is>
       </c>
-      <c r="C29" s="8" t="inlineStr">
+      <c r="C29" s="15" t="inlineStr">
         <is>
           <t>ديمو/وهمية</t>
         </is>
@@ -1782,7 +1864,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="inlineStr">
+      <c r="A30" s="15" t="inlineStr">
         <is>
           <t>ولي الأمر</t>
         </is>
@@ -1792,12 +1874,12 @@
           <t>تقرير الابن</t>
         </is>
       </c>
-      <c r="C30" s="8" t="inlineStr">
+      <c r="C30" s="15" t="inlineStr">
         <is>
           <t>ديمو/وهمية</t>
         </is>
       </c>
-      <c r="D30" s="11" t="inlineStr">
+      <c r="D30" s="16" t="inlineStr">
         <is>
           <t>حقيقية 100%</t>
         </is>
@@ -1819,7 +1901,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+      <c r="A31" s="15" t="inlineStr">
         <is>
           <t>ولي الأمر</t>
         </is>
@@ -1829,12 +1911,12 @@
           <t>الإعدادات</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
+      <c r="C31" s="15" t="inlineStr">
         <is>
           <t>ديمو/وهمية</t>
         </is>
       </c>
-      <c r="D31" s="12" t="inlineStr">
+      <c r="D31" s="17" t="inlineStr">
         <is>
           <t>حقيقية جزئياً (عرض الأبناء فقط)</t>
         </is>
@@ -1899,7 +1981,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>FR-I01</t>
         </is>
@@ -1909,7 +1991,7 @@
           <t>إنشاء كورس حضوري (منشئ المحتوى/المعلم)</t>
         </is>
       </c>
-      <c r="C2" s="12" t="inlineStr">
+      <c r="C2" s="17" t="inlineStr">
         <is>
           <t>🚫 محظور مؤقتاً</t>
         </is>
@@ -1921,7 +2003,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>FR-I02</t>
         </is>
@@ -1931,7 +2013,7 @@
           <t>تهيئة مجموعة طلاب حضورية</t>
         </is>
       </c>
-      <c r="C3" s="12" t="inlineStr">
+      <c r="C3" s="17" t="inlineStr">
         <is>
           <t>🚫 محظور مؤقتاً</t>
         </is>
@@ -1943,7 +2025,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>FR-I03</t>
         </is>
@@ -1953,7 +2035,7 @@
           <t>عرض طلاب المجموعة الحضورية</t>
         </is>
       </c>
-      <c r="C4" s="12" t="inlineStr">
+      <c r="C4" s="17" t="inlineStr">
         <is>
           <t>🚫 محظور مؤقتاً</t>
         </is>
@@ -1965,7 +2047,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>FR-I04</t>
         </is>
@@ -1975,7 +2057,7 @@
           <t>إنشاء وجدولة دروس حضورية</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>🚫 محظور مؤقتاً</t>
         </is>
@@ -1987,7 +2069,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>FR-I05</t>
         </is>
@@ -1997,7 +2079,7 @@
           <t>إنشاء كورس أونلاين</t>
         </is>
       </c>
-      <c r="C6" s="12" t="inlineStr">
+      <c r="C6" s="17" t="inlineStr">
         <is>
           <t>🚫 محظور مؤقتاً</t>
         </is>
@@ -2009,7 +2091,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>FR-I06</t>
         </is>
@@ -2019,7 +2101,7 @@
           <t>تهيئة مجموعة كورس أونلاين</t>
         </is>
       </c>
-      <c r="C7" s="12" t="inlineStr">
+      <c r="C7" s="17" t="inlineStr">
         <is>
           <t>🚫 محظور مؤقتاً</t>
         </is>
@@ -2031,7 +2113,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>FR-I07</t>
         </is>
@@ -2041,7 +2123,7 @@
           <t>تهيئة منصة الاجتماع أونلاين</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="C8" s="17" t="inlineStr">
         <is>
           <t>🚫 محظور مؤقتاً</t>
         </is>
@@ -2053,7 +2135,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>FR-I08</t>
         </is>
@@ -2063,7 +2145,7 @@
           <t>إنشاء وجدولة دروس أونلاين</t>
         </is>
       </c>
-      <c r="C9" s="12" t="inlineStr">
+      <c r="C9" s="17" t="inlineStr">
         <is>
           <t>🚫 محظور مؤقتاً</t>
         </is>
@@ -2075,7 +2157,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>FR-I09</t>
         </is>
@@ -2085,7 +2167,7 @@
           <t>عرض جدول الكورس</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C10" s="17" t="inlineStr">
         <is>
           <t>🚫 محظور مؤقتاً</t>
         </is>
@@ -2097,7 +2179,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>FR-I10</t>
         </is>
@@ -2107,7 +2189,7 @@
           <t>تحديث درس مجدول</t>
         </is>
       </c>
-      <c r="C11" s="12" t="inlineStr">
+      <c r="C11" s="17" t="inlineStr">
         <is>
           <t>🚫 محظور مؤقتاً</t>
         </is>
@@ -2119,7 +2201,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>FR-I11</t>
         </is>
@@ -2129,7 +2211,7 @@
           <t>إلغاء درس مجدول</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
+      <c r="C12" s="17" t="inlineStr">
         <is>
           <t>🚫 محظور مؤقتاً</t>
         </is>
@@ -2141,7 +2223,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>FR-T01</t>
         </is>
@@ -2151,7 +2233,7 @@
           <t>بحث عن معلمين</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
+      <c r="C13" s="16" t="inlineStr">
         <is>
           <t>✅ مطبّق</t>
         </is>
@@ -2163,7 +2245,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>FR-T02</t>
         </is>
@@ -2173,7 +2255,7 @@
           <t>تصفية المعلمين</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="C14" s="16" t="inlineStr">
         <is>
           <t>✅ مطبّق</t>
         </is>
@@ -2185,7 +2267,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>FR-T03</t>
         </is>
@@ -2195,7 +2277,7 @@
           <t>عرض ملف المعلم</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
+      <c r="C15" s="16" t="inlineStr">
         <is>
           <t>✅ مطبّق</t>
         </is>
@@ -2207,7 +2289,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>FR-T04</t>
         </is>
@@ -2217,7 +2299,7 @@
           <t>عرض توفّر المعلم</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C16" s="16" t="inlineStr">
         <is>
           <t>✅ مطبّق</t>
         </is>
@@ -2229,7 +2311,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>FR-T05</t>
         </is>
@@ -2239,7 +2321,7 @@
           <t>إرسال طلب حجز معلم</t>
         </is>
       </c>
-      <c r="C17" s="12" t="inlineStr">
+      <c r="C17" s="17" t="inlineStr">
         <is>
           <t>🚫 محظور بقصد أمني</t>
         </is>
@@ -2251,7 +2333,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="15" t="inlineStr">
         <is>
           <t>FR-T06</t>
         </is>
@@ -2261,7 +2343,7 @@
           <t>معالجة دفع الحجز</t>
         </is>
       </c>
-      <c r="C18" s="12" t="inlineStr">
+      <c r="C18" s="17" t="inlineStr">
         <is>
           <t>🚫 محظور بقصد أمني</t>
         </is>
@@ -2273,7 +2355,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>FR-T07</t>
         </is>
@@ -2283,803 +2365,803 @@
           <t>عرض تقييمات المعلم</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
+      <c r="C19" s="17" t="inlineStr">
+        <is>
+          <t>⚠️ جزئي</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>التقييم الإجمالي (averageRating/ratingCount) موجود ومعروض بملف المعلم؛ نصوص المراجعات بلا endpoint — تُعرض حالة فراغ صادقة</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>FR-T08</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>إدارة ملف المعلم للاكتشاف</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="inlineStr">
+        <is>
+          <t>✅ مطبّق (بتدهور رشيق)</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>teacher.profile.edit.tsx — Teacher/UpdateProfile</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>FR-T09</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>إدارة توفّر المعلم</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>✅ مطبّق (بتدهور رشيق)</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>teacher.settings.tsx — Teacher/SetAvailability</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>FR-T10</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>إدارة طلبات حجز المعلم</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>🚫 محظور بقصد أمني</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>BookingController بلا Authorize (P0-1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>FR-T11</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>تقييم المعلم بعد الجلسة</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>🚫 محظور مؤقتاً</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>Booking/Rate جاهز، غير مربوط</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>FR-W01</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>تقديم طلب شحن محفظة</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>✅ مطبّق</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Student side — Wallet/SubmitTopUpRequest</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>FR-W02</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>التحقق من الشحن واعتماده</t>
+        </is>
+      </c>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>✅ مطبّق</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>admin.payments — Wallet/VerifyTopUpRequest</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t>FR-W04</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>طلب سحب أرباح (معلم)</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="inlineStr">
+        <is>
+          <t>✅ مطبّق</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>teacher.earnings — Wallet/SubmitWithdrawalRequest</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>FR-W06</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>عرض سجل معاملات المحفظة</t>
+        </is>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>✅ مطبّق</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>Wallet/GetTransactionHistory</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>FR-W07</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>تهيئة نسبة عمولة المنصة</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
         <is>
           <t>❌ غير مطبّق بالباك</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
-        <is>
-          <t>لا حقل Rating ظاهر بـPublicProfile حالياً — يحتاج تأكيد إضافي</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t>FR-T08</t>
-        </is>
-      </c>
-      <c r="B20" s="9" t="inlineStr">
-        <is>
-          <t>إدارة ملف المعلم للاكتشاف</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>✅ مطبّق (بتدهور رشيق)</t>
-        </is>
-      </c>
-      <c r="D20" s="9" t="inlineStr">
-        <is>
-          <t>teacher.profile.edit.tsx — Teacher/UpdateProfile</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t>FR-T09</t>
-        </is>
-      </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>إدارة توفّر المعلم</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>✅ مطبّق (بتدهور رشيق)</t>
-        </is>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>teacher.settings.tsx — Teacher/SetAvailability</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>FR-T10</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>إدارة طلبات حجز المعلم</t>
-        </is>
-      </c>
-      <c r="C22" s="12" t="inlineStr">
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>لا endpoint لإعداد نسبة عمولة — يحتاج تأكيد من فريق الباك اند</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>FR-P01</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>الوصول لحساب ولي الأمر</t>
+        </is>
+      </c>
+      <c r="C29" s="16" t="inlineStr">
+        <is>
+          <t>✅ مطبّق</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>تسجيل دخول عادي، UserTypeId=4</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>FR-P02</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>عرض الطلاب المرتبطين</t>
+        </is>
+      </c>
+      <c r="C30" s="18" t="inlineStr">
+        <is>
+          <t>⚠️ مطبّق لكن فاضي دائماً</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>Parent/MyChildren — لا endpoint لربط ابن (FR-P09 غير مطبّق)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>FR-P03</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>عرض نظرة أكاديمية عامة عن الطالب</t>
+        </is>
+      </c>
+      <c r="C31" s="18" t="inlineStr">
+        <is>
+          <t>⚠️ مطبّق لكن فاضي دائماً</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>نفس القيد أعلاه</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="15" t="inlineStr">
+        <is>
+          <t>FR-P04</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>عرض حضور الطالب</t>
+        </is>
+      </c>
+      <c r="C32" s="18" t="inlineStr">
+        <is>
+          <t>⚠️ مطبّق لكن فاضي دائماً</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>Parent/ChildAttendance</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="15" t="inlineStr">
+        <is>
+          <t>FR-P05</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>عرض نتائج امتحانات الطالب</t>
+        </is>
+      </c>
+      <c r="C33" s="18" t="inlineStr">
+        <is>
+          <t>⚠️ مطبّق لكن فاضي دائماً</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>Parent/ChildExamResults</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="15" t="inlineStr">
+        <is>
+          <t>FR-P06</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>حساب نسبة الحضور</t>
+        </is>
+      </c>
+      <c r="C34" s="16" t="inlineStr">
+        <is>
+          <t>✅ مطبّق (بالباك)</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>ضمن ChildOverviewDto</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="15" t="inlineStr">
+        <is>
+          <t>FR-P07</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>حساب متوسط درجات الامتحانات</t>
+        </is>
+      </c>
+      <c r="C35" s="16" t="inlineStr">
+        <is>
+          <t>✅ مطبّق (بالباك)</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
+        <is>
+          <t>ضمن ChildOverviewDto</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="15" t="inlineStr">
+        <is>
+          <t>FR-P08</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>حصر وصول ولي الأمر على أبنائه فقط</t>
+        </is>
+      </c>
+      <c r="C36" s="14" t="inlineStr">
+        <is>
+          <t>⚠️ غير مؤكد</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>ParentController بلا Authorize ظاهر بالكود الخام (P0-1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="15" t="inlineStr">
+        <is>
+          <t>FR-P09</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>ربط ولي أمر بطالب</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="inlineStr">
+        <is>
+          <t>❌ غير مطبّق بالباك</t>
+        </is>
+      </c>
+      <c r="D37" s="9" t="inlineStr">
+        <is>
+          <t>لا Controller/endpoint لهذا إطلاقاً — أهم فجوة بمسار ولي الأمر</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="15" t="inlineStr">
+        <is>
+          <t>FR-P10</t>
+        </is>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>إدارة نوع علاقة الوصاية</t>
+        </is>
+      </c>
+      <c r="C38" s="10" t="inlineStr">
+        <is>
+          <t>❌ غير مطبّق بالباك</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>مرتبط بـFR-P09</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="15" t="inlineStr">
+        <is>
+          <t>FR-P11</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>عرض إشعارات ولي الأمر</t>
+        </is>
+      </c>
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>❌ غير مطبّق بالباك</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>لا endpoint إشعارات لغير الطالب</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="15" t="inlineStr">
+        <is>
+          <t>FR-P12</t>
+        </is>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>فرض قراءة فقط بالمتابعة الأكاديمية</t>
+        </is>
+      </c>
+      <c r="C40" s="16" t="inlineStr">
+        <is>
+          <t>✅ مطبّق بالتصميم</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>Parent Controller GET فقط، لا كتابة</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="15" t="inlineStr">
+        <is>
+          <t>FR-P13</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>عرض اسم وصف الطالب</t>
+        </is>
+      </c>
+      <c r="C41" s="18" t="inlineStr">
+        <is>
+          <t>⚠️ مطبّق لكن فاضي دائماً</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>ضمن نفس قيد FR-P02</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="15" t="inlineStr">
+        <is>
+          <t>FR-S01</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>عرض لوحة الطالب</t>
+        </is>
+      </c>
+      <c r="C42" s="16" t="inlineStr">
+        <is>
+          <t>✅ مطبّق</t>
+        </is>
+      </c>
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>Student/Dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="15" t="inlineStr">
+        <is>
+          <t>FR-S02</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>عرض طلبات الحجز</t>
+        </is>
+      </c>
+      <c r="C43" s="16" t="inlineStr">
+        <is>
+          <t>✅ مطبّق</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>Student/MyRequests</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="15" t="inlineStr">
+        <is>
+          <t>FR-S03</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>عرض حالة الحجز</t>
+        </is>
+      </c>
+      <c r="C44" s="16" t="inlineStr">
+        <is>
+          <t>✅ مطبّق</t>
+        </is>
+      </c>
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>ضمن MyRequests/MyBookings</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="15" t="inlineStr">
+        <is>
+          <t>FR-S04</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>عرض الحجوزات المؤكّدة</t>
+        </is>
+      </c>
+      <c r="C45" s="16" t="inlineStr">
+        <is>
+          <t>✅ مطبّق</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>Student/MyBookings</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="15" t="inlineStr">
+        <is>
+          <t>FR-S05</t>
+        </is>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>عرض جدول الطالب</t>
+        </is>
+      </c>
+      <c r="C46" s="16" t="inlineStr">
+        <is>
+          <t>✅ مطبّق</t>
+        </is>
+      </c>
+      <c r="D46" s="9" t="inlineStr">
+        <is>
+          <t>Student/Schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="15" t="inlineStr">
+        <is>
+          <t>FR-S06</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>عرض معلومات درس حضوري</t>
+        </is>
+      </c>
+      <c r="C47" s="16" t="inlineStr">
+        <is>
+          <t>✅ مطبّق</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>ضمن Schedule/MyBookings</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="15" t="inlineStr">
+        <is>
+          <t>FR-S07</t>
+        </is>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>عرض معلومات درس أونلاين</t>
+        </is>
+      </c>
+      <c r="C48" s="16" t="inlineStr">
+        <is>
+          <t>✅ مطبّق</t>
+        </is>
+      </c>
+      <c r="D48" s="9" t="inlineStr">
+        <is>
+          <t>ضمن Schedule/MyBookings (رابط الاجتماع)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="15" t="inlineStr">
+        <is>
+          <t>FR-S08</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>عرض تفاصيل كورس ودرس</t>
+        </is>
+      </c>
+      <c r="C49" s="16" t="inlineStr">
+        <is>
+          <t>✅ مطبّق</t>
+        </is>
+      </c>
+      <c r="D49" s="9" t="inlineStr">
+        <is>
+          <t>Student/GetCourse, GetLesson</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="15" t="inlineStr">
+        <is>
+          <t>FR-S09</t>
+        </is>
+      </c>
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>عرض حضور الطالب</t>
+        </is>
+      </c>
+      <c r="C50" s="16" t="inlineStr">
+        <is>
+          <t>✅ مطبّق</t>
+        </is>
+      </c>
+      <c r="D50" s="9" t="inlineStr">
+        <is>
+          <t>Student/Attendance</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="15" t="inlineStr">
+        <is>
+          <t>FR-S10</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>عرض نتائج الامتحانات</t>
+        </is>
+      </c>
+      <c r="C51" s="16" t="inlineStr">
+        <is>
+          <t>✅ مطبّق</t>
+        </is>
+      </c>
+      <c r="D51" s="9" t="inlineStr">
+        <is>
+          <t>Student/ExamResults</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="15" t="inlineStr">
+        <is>
+          <t>FR-S11</t>
+        </is>
+      </c>
+      <c r="B52" s="9" t="inlineStr">
+        <is>
+          <t>عرض التقدّم الأكاديمي</t>
+        </is>
+      </c>
+      <c r="C52" s="16" t="inlineStr">
+        <is>
+          <t>✅ مطبّق</t>
+        </is>
+      </c>
+      <c r="D52" s="9" t="inlineStr">
+        <is>
+          <t>Student/Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="15" t="inlineStr">
+        <is>
+          <t>FR-S12</t>
+        </is>
+      </c>
+      <c r="B53" s="9" t="inlineStr">
+        <is>
+          <t>عرض إشعارات الطالب</t>
+        </is>
+      </c>
+      <c r="C53" s="16" t="inlineStr">
+        <is>
+          <t>✅ مطبّق</t>
+        </is>
+      </c>
+      <c r="D53" s="9" t="inlineStr">
+        <is>
+          <t>Student/Notifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="15" t="inlineStr">
+        <is>
+          <t>FR-S13</t>
+        </is>
+      </c>
+      <c r="B54" s="9" t="inlineStr">
+        <is>
+          <t>عرض معلومات محفظة الطالب</t>
+        </is>
+      </c>
+      <c r="C54" s="16" t="inlineStr">
+        <is>
+          <t>✅ مطبّق</t>
+        </is>
+      </c>
+      <c r="D54" s="9" t="inlineStr">
+        <is>
+          <t>Wallet/MyWallet</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="15" t="inlineStr">
+        <is>
+          <t>FR-S14</t>
+        </is>
+      </c>
+      <c r="B55" s="9" t="inlineStr">
+        <is>
+          <t>إلغاء حجز الطالب</t>
+        </is>
+      </c>
+      <c r="C55" s="17" t="inlineStr">
         <is>
           <t>🚫 محظور بقصد أمني</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>BookingController بلا Authorize (P0-1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="8" t="inlineStr">
-        <is>
-          <t>FR-T11</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>تقييم المعلم بعد الجلسة</t>
-        </is>
-      </c>
-      <c r="C23" s="12" t="inlineStr">
-        <is>
-          <t>🚫 محظور مؤقتاً</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>Booking/Rate جاهز، غير مربوط</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="8" t="inlineStr">
-        <is>
-          <t>FR-W01</t>
-        </is>
-      </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>تقديم طلب شحن محفظة</t>
-        </is>
-      </c>
-      <c r="C24" s="11" t="inlineStr">
-        <is>
-          <t>✅ مطبّق</t>
-        </is>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>Student side — Wallet/SubmitTopUpRequest</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="8" t="inlineStr">
-        <is>
-          <t>FR-W02</t>
-        </is>
-      </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>التحقق من الشحن واعتماده</t>
-        </is>
-      </c>
-      <c r="C25" s="11" t="inlineStr">
-        <is>
-          <t>✅ مطبّق</t>
-        </is>
-      </c>
-      <c r="D25" s="9" t="inlineStr">
-        <is>
-          <t>admin.payments — Wallet/VerifyTopUpRequest</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="8" t="inlineStr">
-        <is>
-          <t>FR-W04</t>
-        </is>
-      </c>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>طلب سحب أرباح (معلم)</t>
-        </is>
-      </c>
-      <c r="C26" s="11" t="inlineStr">
-        <is>
-          <t>✅ مطبّق</t>
-        </is>
-      </c>
-      <c r="D26" s="9" t="inlineStr">
-        <is>
-          <t>teacher.earnings — Wallet/SubmitWithdrawalRequest</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="8" t="inlineStr">
-        <is>
-          <t>FR-W06</t>
-        </is>
-      </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>عرض سجل معاملات المحفظة</t>
-        </is>
-      </c>
-      <c r="C27" s="11" t="inlineStr">
-        <is>
-          <t>✅ مطبّق</t>
-        </is>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
-        <is>
-          <t>Wallet/GetTransactionHistory</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
-        <is>
-          <t>FR-W07</t>
-        </is>
-      </c>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>تهيئة نسبة عمولة المنصة</t>
-        </is>
-      </c>
-      <c r="C28" s="10" t="inlineStr">
-        <is>
-          <t>❌ غير مطبّق بالباك</t>
-        </is>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
-        <is>
-          <t>لا endpoint لإعداد نسبة عمولة — يحتاج تأكيد من فريق الباك اند</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="8" t="inlineStr">
-        <is>
-          <t>FR-P01</t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>الوصول لحساب ولي الأمر</t>
-        </is>
-      </c>
-      <c r="C29" s="11" t="inlineStr">
-        <is>
-          <t>✅ مطبّق</t>
-        </is>
-      </c>
-      <c r="D29" s="9" t="inlineStr">
-        <is>
-          <t>تسجيل دخول عادي، UserTypeId=4</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t>FR-P02</t>
-        </is>
-      </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>عرض الطلاب المرتبطين</t>
-        </is>
-      </c>
-      <c r="C30" s="13" t="inlineStr">
-        <is>
-          <t>⚠️ مطبّق لكن فاضي دائماً</t>
-        </is>
-      </c>
-      <c r="D30" s="9" t="inlineStr">
-        <is>
-          <t>Parent/MyChildren — لا endpoint لربط ابن (FR-P09 غير مطبّق)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t>FR-P03</t>
-        </is>
-      </c>
-      <c r="B31" s="9" t="inlineStr">
-        <is>
-          <t>عرض نظرة أكاديمية عامة عن الطالب</t>
-        </is>
-      </c>
-      <c r="C31" s="13" t="inlineStr">
-        <is>
-          <t>⚠️ مطبّق لكن فاضي دائماً</t>
-        </is>
-      </c>
-      <c r="D31" s="9" t="inlineStr">
-        <is>
-          <t>نفس القيد أعلاه</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr">
-        <is>
-          <t>FR-P04</t>
-        </is>
-      </c>
-      <c r="B32" s="9" t="inlineStr">
-        <is>
-          <t>عرض حضور الطالب</t>
-        </is>
-      </c>
-      <c r="C32" s="13" t="inlineStr">
-        <is>
-          <t>⚠️ مطبّق لكن فاضي دائماً</t>
-        </is>
-      </c>
-      <c r="D32" s="9" t="inlineStr">
-        <is>
-          <t>Parent/ChildAttendance</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
-        <is>
-          <t>FR-P05</t>
-        </is>
-      </c>
-      <c r="B33" s="9" t="inlineStr">
-        <is>
-          <t>عرض نتائج امتحانات الطالب</t>
-        </is>
-      </c>
-      <c r="C33" s="13" t="inlineStr">
-        <is>
-          <t>⚠️ مطبّق لكن فاضي دائماً</t>
-        </is>
-      </c>
-      <c r="D33" s="9" t="inlineStr">
-        <is>
-          <t>Parent/ChildExamResults</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="8" t="inlineStr">
-        <is>
-          <t>FR-P06</t>
-        </is>
-      </c>
-      <c r="B34" s="9" t="inlineStr">
-        <is>
-          <t>حساب نسبة الحضور</t>
-        </is>
-      </c>
-      <c r="C34" s="11" t="inlineStr">
-        <is>
-          <t>✅ مطبّق (بالباك)</t>
-        </is>
-      </c>
-      <c r="D34" s="9" t="inlineStr">
-        <is>
-          <t>ضمن ChildOverviewDto</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
-        <is>
-          <t>FR-P07</t>
-        </is>
-      </c>
-      <c r="B35" s="9" t="inlineStr">
-        <is>
-          <t>حساب متوسط درجات الامتحانات</t>
-        </is>
-      </c>
-      <c r="C35" s="11" t="inlineStr">
-        <is>
-          <t>✅ مطبّق (بالباك)</t>
-        </is>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
-        <is>
-          <t>ضمن ChildOverviewDto</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
-        <is>
-          <t>FR-P08</t>
-        </is>
-      </c>
-      <c r="B36" s="9" t="inlineStr">
-        <is>
-          <t>حصر وصول ولي الأمر على أبنائه فقط</t>
-        </is>
-      </c>
-      <c r="C36" s="14" t="inlineStr">
-        <is>
-          <t>⚠️ غير مؤكد</t>
-        </is>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
-        <is>
-          <t>ParentController بلا Authorize ظاهر بالكود الخام (P0-1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
-        <is>
-          <t>FR-P09</t>
-        </is>
-      </c>
-      <c r="B37" s="9" t="inlineStr">
-        <is>
-          <t>ربط ولي أمر بطالب</t>
-        </is>
-      </c>
-      <c r="C37" s="10" t="inlineStr">
-        <is>
-          <t>❌ غير مطبّق بالباك</t>
-        </is>
-      </c>
-      <c r="D37" s="9" t="inlineStr">
-        <is>
-          <t>لا Controller/endpoint لهذا إطلاقاً — أهم فجوة بمسار ولي الأمر</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
-        <is>
-          <t>FR-P10</t>
-        </is>
-      </c>
-      <c r="B38" s="9" t="inlineStr">
-        <is>
-          <t>إدارة نوع علاقة الوصاية</t>
-        </is>
-      </c>
-      <c r="C38" s="10" t="inlineStr">
-        <is>
-          <t>❌ غير مطبّق بالباك</t>
-        </is>
-      </c>
-      <c r="D38" s="9" t="inlineStr">
-        <is>
-          <t>مرتبط بـFR-P09</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
-        <is>
-          <t>FR-P11</t>
-        </is>
-      </c>
-      <c r="B39" s="9" t="inlineStr">
-        <is>
-          <t>عرض إشعارات ولي الأمر</t>
-        </is>
-      </c>
-      <c r="C39" s="10" t="inlineStr">
-        <is>
-          <t>❌ غير مطبّق بالباك</t>
-        </is>
-      </c>
-      <c r="D39" s="9" t="inlineStr">
-        <is>
-          <t>لا endpoint إشعارات لغير الطالب</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
-        <is>
-          <t>FR-P12</t>
-        </is>
-      </c>
-      <c r="B40" s="9" t="inlineStr">
-        <is>
-          <t>فرض قراءة فقط بالمتابعة الأكاديمية</t>
-        </is>
-      </c>
-      <c r="C40" s="11" t="inlineStr">
-        <is>
-          <t>✅ مطبّق بالتصميم</t>
-        </is>
-      </c>
-      <c r="D40" s="9" t="inlineStr">
-        <is>
-          <t>Parent Controller GET فقط، لا كتابة</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
-        <is>
-          <t>FR-P13</t>
-        </is>
-      </c>
-      <c r="B41" s="9" t="inlineStr">
-        <is>
-          <t>عرض اسم وصف الطالب</t>
-        </is>
-      </c>
-      <c r="C41" s="13" t="inlineStr">
-        <is>
-          <t>⚠️ مطبّق لكن فاضي دائماً</t>
-        </is>
-      </c>
-      <c r="D41" s="9" t="inlineStr">
-        <is>
-          <t>ضمن نفس قيد FR-P02</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="8" t="inlineStr">
-        <is>
-          <t>FR-S01</t>
-        </is>
-      </c>
-      <c r="B42" s="9" t="inlineStr">
-        <is>
-          <t>عرض لوحة الطالب</t>
-        </is>
-      </c>
-      <c r="C42" s="11" t="inlineStr">
-        <is>
-          <t>✅ مطبّق</t>
-        </is>
-      </c>
-      <c r="D42" s="9" t="inlineStr">
-        <is>
-          <t>Student/Dashboard</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
-        <is>
-          <t>FR-S02</t>
-        </is>
-      </c>
-      <c r="B43" s="9" t="inlineStr">
-        <is>
-          <t>عرض طلبات الحجز</t>
-        </is>
-      </c>
-      <c r="C43" s="11" t="inlineStr">
-        <is>
-          <t>✅ مطبّق</t>
-        </is>
-      </c>
-      <c r="D43" s="9" t="inlineStr">
-        <is>
-          <t>Student/MyRequests</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
-        <is>
-          <t>FR-S03</t>
-        </is>
-      </c>
-      <c r="B44" s="9" t="inlineStr">
-        <is>
-          <t>عرض حالة الحجز</t>
-        </is>
-      </c>
-      <c r="C44" s="11" t="inlineStr">
-        <is>
-          <t>✅ مطبّق</t>
-        </is>
-      </c>
-      <c r="D44" s="9" t="inlineStr">
-        <is>
-          <t>ضمن MyRequests/MyBookings</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
-        <is>
-          <t>FR-S04</t>
-        </is>
-      </c>
-      <c r="B45" s="9" t="inlineStr">
-        <is>
-          <t>عرض الحجوزات المؤكّدة</t>
-        </is>
-      </c>
-      <c r="C45" s="11" t="inlineStr">
-        <is>
-          <t>✅ مطبّق</t>
-        </is>
-      </c>
-      <c r="D45" s="9" t="inlineStr">
-        <is>
-          <t>Student/MyBookings</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="inlineStr">
-        <is>
-          <t>FR-S05</t>
-        </is>
-      </c>
-      <c r="B46" s="9" t="inlineStr">
-        <is>
-          <t>عرض جدول الطالب</t>
-        </is>
-      </c>
-      <c r="C46" s="11" t="inlineStr">
-        <is>
-          <t>✅ مطبّق</t>
-        </is>
-      </c>
-      <c r="D46" s="9" t="inlineStr">
-        <is>
-          <t>Student/Schedule</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
-        <is>
-          <t>FR-S06</t>
-        </is>
-      </c>
-      <c r="B47" s="9" t="inlineStr">
-        <is>
-          <t>عرض معلومات درس حضوري</t>
-        </is>
-      </c>
-      <c r="C47" s="11" t="inlineStr">
-        <is>
-          <t>✅ مطبّق</t>
-        </is>
-      </c>
-      <c r="D47" s="9" t="inlineStr">
-        <is>
-          <t>ضمن Schedule/MyBookings</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
-        <is>
-          <t>FR-S07</t>
-        </is>
-      </c>
-      <c r="B48" s="9" t="inlineStr">
-        <is>
-          <t>عرض معلومات درس أونلاين</t>
-        </is>
-      </c>
-      <c r="C48" s="11" t="inlineStr">
-        <is>
-          <t>✅ مطبّق</t>
-        </is>
-      </c>
-      <c r="D48" s="9" t="inlineStr">
-        <is>
-          <t>ضمن Schedule/MyBookings (رابط الاجتماع)</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="8" t="inlineStr">
-        <is>
-          <t>FR-S08</t>
-        </is>
-      </c>
-      <c r="B49" s="9" t="inlineStr">
-        <is>
-          <t>عرض تفاصيل كورس ودرس</t>
-        </is>
-      </c>
-      <c r="C49" s="11" t="inlineStr">
-        <is>
-          <t>✅ مطبّق</t>
-        </is>
-      </c>
-      <c r="D49" s="9" t="inlineStr">
-        <is>
-          <t>Student/GetCourse, GetLesson</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
-        <is>
-          <t>FR-S09</t>
-        </is>
-      </c>
-      <c r="B50" s="9" t="inlineStr">
-        <is>
-          <t>عرض حضور الطالب</t>
-        </is>
-      </c>
-      <c r="C50" s="11" t="inlineStr">
-        <is>
-          <t>✅ مطبّق</t>
-        </is>
-      </c>
-      <c r="D50" s="9" t="inlineStr">
-        <is>
-          <t>Student/Attendance</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr">
-        <is>
-          <t>FR-S10</t>
-        </is>
-      </c>
-      <c r="B51" s="9" t="inlineStr">
-        <is>
-          <t>عرض نتائج الامتحانات</t>
-        </is>
-      </c>
-      <c r="C51" s="11" t="inlineStr">
-        <is>
-          <t>✅ مطبّق</t>
-        </is>
-      </c>
-      <c r="D51" s="9" t="inlineStr">
-        <is>
-          <t>Student/ExamResults</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="8" t="inlineStr">
-        <is>
-          <t>FR-S11</t>
-        </is>
-      </c>
-      <c r="B52" s="9" t="inlineStr">
-        <is>
-          <t>عرض التقدّم الأكاديمي</t>
-        </is>
-      </c>
-      <c r="C52" s="11" t="inlineStr">
-        <is>
-          <t>✅ مطبّق</t>
-        </is>
-      </c>
-      <c r="D52" s="9" t="inlineStr">
-        <is>
-          <t>Student/Progress</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="8" t="inlineStr">
-        <is>
-          <t>FR-S12</t>
-        </is>
-      </c>
-      <c r="B53" s="9" t="inlineStr">
-        <is>
-          <t>عرض إشعارات الطالب</t>
-        </is>
-      </c>
-      <c r="C53" s="11" t="inlineStr">
-        <is>
-          <t>✅ مطبّق</t>
-        </is>
-      </c>
-      <c r="D53" s="9" t="inlineStr">
-        <is>
-          <t>Student/Notifications</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="8" t="inlineStr">
-        <is>
-          <t>FR-S13</t>
-        </is>
-      </c>
-      <c r="B54" s="9" t="inlineStr">
-        <is>
-          <t>عرض معلومات محفظة الطالب</t>
-        </is>
-      </c>
-      <c r="C54" s="11" t="inlineStr">
-        <is>
-          <t>✅ مطبّق</t>
-        </is>
-      </c>
-      <c r="D54" s="9" t="inlineStr">
-        <is>
-          <t>Wallet/MyWallet</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="inlineStr">
-        <is>
-          <t>FR-S14</t>
-        </is>
-      </c>
-      <c r="B55" s="9" t="inlineStr">
-        <is>
-          <t>إلغاء حجز الطالب</t>
-        </is>
-      </c>
-      <c r="C55" s="12" t="inlineStr">
-        <is>
-          <t>🚫 محظور بقصد أمني</t>
-        </is>
-      </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
           <t>Student/CancelBooking جاهز — غير مربوط (يعتمد على Booking الآمن)</t>
@@ -3087,7 +3169,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="8" t="inlineStr">
+      <c r="A56" s="15" t="inlineStr">
         <is>
           <t>FR-S15</t>
         </is>
@@ -3097,7 +3179,7 @@
           <t>طلب إعادة جدولة حجز</t>
         </is>
       </c>
-      <c r="C56" s="12" t="inlineStr">
+      <c r="C56" s="17" t="inlineStr">
         <is>
           <t>🚫 محظور بقصد أمني</t>
         </is>
@@ -3524,25 +3606,25 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="45" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+    <row r="2" ht="60" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>UserTypeIds</t>
         </is>
       </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
-          <t>الأرقام بالكود (Admin=1,Student=3,Teacher=4,Parent=5) لا تطابق البيانات المزروعة فعلياً (1,2,3,4) — فرق كامل بالترقيم.</t>
+          <t>تم اعتماد القرار: تُعاد كتابة UserSeed.cs لتطابق ثابت الكود (Admin=1, Student=3, Teacher=4, Parent=5 — رقم 2 محجوز). الفرونت اند عُدّل بالكامل ليطابق (admin-dashboard.tsx).</t>
         </is>
       </c>
       <c r="C2" s="9" t="inlineStr">
         <is>
-          <t>أي [RequireUserTypes] حالي كان بيرفض كل مستخدم حقيقي (طالب حقيقي يتحقق كأنه معلم وبالعكس).</t>
-        </is>
-      </c>
-      <c r="D2" s="19" t="inlineStr">
-        <is>
-          <t>✅ تم الاتفاق على التصحيح — الفريق هيعتمد 1,2,3,4</t>
+          <t>⚠️ التعديل بملف UserSeed.cs وحده لا يكفي — القيم Baked بميغريشن EF Core سابقة. لازم Migration جديدة فيها UPDATE صريح لأي صفوف موجودة فعلياً + أي FK عليها (Users.UserTypeId وغيرها) — وإلا التعديل ما رح ينعكس على قاعدة بيانات شغّالة.</t>
+        </is>
+      </c>
+      <c r="D2" s="20" t="inlineStr">
+        <is>
+          <t>⏳ الكود جاهز كمرجع — بانتظار Migration فعلية من فريق الباك اند</t>
         </is>
       </c>
     </row>
@@ -3763,14 +3845,14 @@
           <t>✅ مطابق 100%</t>
         </is>
       </c>
-      <c r="E3" s="22" t="inlineStr">
-        <is>
-          <t>➖ غير موجودة</t>
+      <c r="E3" s="19" t="inlineStr">
+        <is>
+          <t>✅ أُضيفت</t>
         </is>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>حجم الجدول محدود طبيعياً (صفحات نظام)، أولوية منخفضة</t>
+          <t>Pagination من جهة الفرونت (البيانات كلها محمّلة أصلاً دفعة وحدة، pageSize=20 بالعرض)</t>
         </is>
       </c>
     </row>
@@ -3859,14 +3941,14 @@
           <t>✅ مطابق 100%</t>
         </is>
       </c>
-      <c r="E6" s="21" t="inlineStr">
-        <is>
-          <t>❌ غير موجودة</t>
+      <c r="E6" s="19" t="inlineStr">
+        <is>
+          <t>✅ أُضيفت</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>الطلبات المعلّقة فقط تُعرض — تتراكم لو الأدمن ما عالجها بانتظام، يُنصح بإضافتها</t>
+          <t>Pagination من جهة الفرونت لكلا القسمين (شحن/سحب) — الباك اند نفسه ما بيدعم skip/pageSize لهالـ2 endpoint</t>
         </is>
       </c>
     </row>
@@ -4002,4 +4084,464 @@
   <autoFilter ref="A1:F10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="23" t="inlineStr">
+        <is>
+          <t>الصفحة</t>
+        </is>
+      </c>
+      <c r="B1" s="23" t="inlineStr">
+        <is>
+          <t>الحالة قبل</t>
+        </is>
+      </c>
+      <c r="C1" s="23" t="inlineStr">
+        <is>
+          <t>الإجراء</t>
+        </is>
+      </c>
+      <c r="D1" s="23" t="inlineStr">
+        <is>
+          <t>الحالة بعد</t>
+        </is>
+      </c>
+      <c r="E1" s="23" t="inlineStr">
+        <is>
+          <t>ملاحظات</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>/teachers , /teacher/$id</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>حقيقية (Teacher/Search, PublicProfile, Availability)</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>فُحصت بنفسي</t>
+        </is>
+      </c>
+      <c r="D2" s="19" t="inlineStr">
+        <is>
+          <t>حقيقية</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>التقييم الإجمالي حقيقي؛ المراجعات النصية حالة فراغ صادقة</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="42" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>/courses , /course/$id</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>حقيقية (Course/GetPublished)</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>فُحصت بنفسي</t>
+        </is>
+      </c>
+      <c r="D3" s="19" t="inlineStr">
+        <is>
+          <t>حقيقية</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr"/>
+    </row>
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>الرئيسية /</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>نصوص تسويقية لمنتج آخر (مكتبة، بطاقات، محاكي، بنك أخطاء، مجتمع)</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>إعادة كتابة كاملة ar/en + معاينة الهيرو بلا أرقام مختلقة</t>
+        </is>
+      </c>
+      <c r="D4" s="19" t="inlineStr">
+        <is>
+          <t>مطابقة للـSRS</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>الأقسام تبقى بنفس مفاتيح i18n لتفادي كسر الكود</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>كيف تعمل /how-it-works</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>وعود ميزات غير موجودة</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>إعادة كتابة</t>
+        </is>
+      </c>
+      <c r="D5" s="19" t="inlineStr">
+        <is>
+          <t>مطابقة</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr"/>
+    </row>
+    <row r="6" ht="42" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>لأولياء الأمور /for-parents</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>تقرير أسبوعي وتنبيهات فورية غير موجودة</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>إعادة كتابة + تنبيه صريح أن الربط والإشعارات قيد التطوير</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>مطابقة</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr"/>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>للمعلمين /for-teachers</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>توثيق وثائق وتحليلات وشارات</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>إعادة كتابة (ملف، توفّر، أرباح، ظهور بالدليل)</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>مطابقة</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr"/>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>من نحن /about , المساعدة /help</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>نصوص عن ميزات محذوفة</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>إعادة كتابة</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>مطابقة</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr"/>
+    </row>
+    <row r="9" ht="42" customHeight="1">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>تسجيل معلّم /teacher/register</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>حقول وثيقة/تخصص/خبرة تُعرض ولا تُرسل</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>إزالة نصوصها غير المستخدمة</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>مطابقة</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>الباك اند يستقبل بيانات التسجيل الأساسية فقط</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>/contact</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>إرسال وهمي (يعرض نجاحاً بلا إرسال)</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>استبداله بفتح بريد mailto جاهز + نص صادق</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="inlineStr">
+        <is>
+          <t>صادقة</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>لا يوجد endpoint تواصل بالباك اند</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>/pricing</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>خطط أسعار وهمية (مجاني/بريميوم)</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>حذف الصفحة والروابط والترجمات</t>
+        </is>
+      </c>
+      <c r="D11" s="21" t="inlineStr">
+        <is>
+          <t>محذوفة</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>لا خطط اشتراك بالـSRS ولا بالباك اند (المحفظة والعمولة فقط)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>/certificate/$id</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>تحقق شهادات وهمي</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>حذف</t>
+        </is>
+      </c>
+      <c r="D12" s="21" t="inlineStr">
+        <is>
+          <t>محذوفة</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>لا كيان Certificate بالباك اند</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>/unsubscribe</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>إلغاء اشتراك وهمي</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>حذف</t>
+        </is>
+      </c>
+      <c r="D13" s="21" t="inlineStr">
+        <is>
+          <t>محذوفة</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>لا نظام نشرة بريدية</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>/invite/$code</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>إحالات وهمية</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>حذف + إزالة باراميتر invite من signup</t>
+        </is>
+      </c>
+      <c r="D14" s="21" t="inlineStr">
+        <is>
+          <t>محذوفة</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>لا نظام إحالات</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="42" customHeight="1">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>/forgot-password , /reset-password , /verify-email</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>نماذج تنتهي دائماً برسالة خطأ</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>حذف + إزالة رابط 'نسيت كلمة المرور' من الدخول</t>
+        </is>
+      </c>
+      <c r="D15" s="21" t="inlineStr">
+        <is>
+          <t>محذوفة</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>لا endpoints لها بالباك اند (Auth: Login/Register/Logout فقط). ChangePassword موجود للمسجّلين — غير مربوط بواجهة بعد</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="42" customHeight="1">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>/blog</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>محتوى تحريري أصلي (نصائح دراسة)</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>لم يُمس</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>سليمة</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>تأكد فريق المحتوى أنه يناسب هوية المنصة</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="42" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>/privacy , /terms</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>نص قانوني</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>تعديل بند الأدوار (حذف المشرف)</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>سليمة</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>مراجعة قانونية مطلوبة قبل النشر</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(plan): update demo cleanup tracking spreadsheet
</commit_message>
<xml_diff>
--- a/Shared/academia-demo-cleanup-plan.xlsx
+++ b/Shared/academia-demo-cleanup-plan.xlsx
@@ -763,10 +763,10 @@
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A23:F23"/>
     <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A22:F22"/>
     <mergeCell ref="A26:F26"/>
-    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A21:F21"/>
     <mergeCell ref="A20:F20"/>
-    <mergeCell ref="A21:F21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3537,7 +3537,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Wallet</t>
         </is>
@@ -3547,19 +3547,19 @@
           <t>MyWallet, GetTransactionHistory, SubmitTopUpRequest, SubmitWithdrawalRequest, GetPendingTopUpRequests, GetPendingWithdrawalRequests, VerifyTopUpRequest, DecideWithdrawalRequest, CompleteWithdrawal, GetReceiptImage</t>
         </is>
       </c>
-      <c r="C13" s="18" t="inlineStr">
-        <is>
-          <t>⚠️ جزئي</t>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>✅ نعم</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>wallet.ts — كل شي مربوط ما عدا CompleteWithdrawal وGetReceiptImage</t>
+          <t>wallet.ts — كل الدوال العشرة مربوطة فعلياً، بما فيها CompleteWithdrawal وGetReceiptImage (تأكدت بالكود، تصحيح لملاحظة سابقة)</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>الاثنين هدول غير مستخدمين حالياً بأي واجهة</t>
+          <t>—</t>
         </is>
       </c>
     </row>

</xml_diff>